<commit_message>
Update IRT prerequisites workbook
</commit_message>
<xml_diff>
--- a/math_question_irt_with_prerequisites.xlsx
+++ b/math_question_irt_with_prerequisites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10705"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/naoki_takahashi/Documents/GitHub/Math_Prompt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{45FE7400-8A35-164D-AA32-EB348A995148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD585F6B-7FD8-B840-90AD-1777847A7D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6220" yWindow="-18500" windowWidth="35340" windowHeight="14660" xr2:uid="{FC93BE12-625C-BB4C-8363-0AA2047E1AA3}"/>
+    <workbookView xWindow="0" yWindow="-18500" windowWidth="35340" windowHeight="14660" xr2:uid="{FC93BE12-625C-BB4C-8363-0AA2047E1AA3}"/>
   </bookViews>
   <sheets>
     <sheet name="math_question_irt_with_prerequi" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">math_question_irt_with_prerequi!$A:$AB</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -3259,7 +3272,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3267,9 +3280,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3647,9 +3657,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D504C1-10AA-394B-B3F6-5620CD148B80}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AB534"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" zeroHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -3657,8 +3666,8 @@
     <col min="6" max="6" width="9" customWidth="1"/>
     <col min="7" max="21" width="10.7109375" hidden="1" customWidth="1"/>
     <col min="22" max="26" width="10.7109375" customWidth="1"/>
-    <col min="27" max="27" width="45.7109375" customWidth="1"/>
-    <col min="28" max="28" width="47.28515625" customWidth="1"/>
+    <col min="27" max="27" width="45.7109375" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="47.28515625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -3747,7 +3756,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:28" hidden="1">
+    <row r="2" spans="1:28">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -3825,7 +3834,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:28" hidden="1">
+    <row r="3" spans="1:28">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -4059,7 +4068,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:28" hidden="1">
+    <row r="6" spans="1:28">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -4143,7 +4152,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:28" hidden="1">
+    <row r="7" spans="1:28">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -4227,7 +4236,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:28" hidden="1">
+    <row r="8" spans="1:28">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -4311,7 +4320,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:28" hidden="1">
+    <row r="9" spans="1:28">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -4395,7 +4404,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:28" hidden="1">
+    <row r="10" spans="1:28">
       <c r="A10" t="s">
         <v>52</v>
       </c>
@@ -4479,7 +4488,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:28" hidden="1">
+    <row r="11" spans="1:28">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -4563,7 +4572,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:28" hidden="1">
+    <row r="12" spans="1:28">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -4647,7 +4656,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:28" hidden="1">
+    <row r="13" spans="1:28">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -4731,7 +4740,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:28" hidden="1">
+    <row r="14" spans="1:28">
       <c r="A14" t="s">
         <v>64</v>
       </c>
@@ -4815,7 +4824,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:28" hidden="1">
+    <row r="15" spans="1:28">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -4899,7 +4908,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:28" hidden="1">
+    <row r="16" spans="1:28">
       <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
@@ -4983,7 +4992,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:28" hidden="1">
+    <row r="17" spans="1:28">
       <c r="A17" s="2" t="s">
         <v>68</v>
       </c>
@@ -5067,7 +5076,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:28" hidden="1">
+    <row r="18" spans="1:28">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -5151,7 +5160,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:28" hidden="1">
+    <row r="19" spans="1:28">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -5235,7 +5244,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:28" hidden="1">
+    <row r="20" spans="1:28">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -5319,7 +5328,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:28" hidden="1">
+    <row r="21" spans="1:28">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -5403,7 +5412,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:28" hidden="1">
+    <row r="22" spans="1:28">
       <c r="A22" s="2" t="s">
         <v>74</v>
       </c>
@@ -5487,7 +5496,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:28" hidden="1">
+    <row r="23" spans="1:28">
       <c r="A23" t="s">
         <v>76</v>
       </c>
@@ -5571,7 +5580,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:28" hidden="1">
+    <row r="24" spans="1:28">
       <c r="A24" t="s">
         <v>77</v>
       </c>
@@ -5655,7 +5664,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:28" hidden="1">
+    <row r="25" spans="1:28">
       <c r="A25" s="2" t="s">
         <v>81</v>
       </c>
@@ -5739,7 +5748,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:28" hidden="1">
+    <row r="26" spans="1:28">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -5823,7 +5832,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:28" hidden="1">
+    <row r="27" spans="1:28">
       <c r="A27" t="s">
         <v>83</v>
       </c>
@@ -5907,7 +5916,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:28" hidden="1">
+    <row r="28" spans="1:28">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -5991,7 +6000,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:28" hidden="1">
+    <row r="29" spans="1:28">
       <c r="A29" s="2" t="s">
         <v>87</v>
       </c>
@@ -6075,7 +6084,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:28" hidden="1">
+    <row r="30" spans="1:28">
       <c r="A30" s="2" t="s">
         <v>88</v>
       </c>
@@ -6159,7 +6168,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:28" hidden="1">
+    <row r="31" spans="1:28">
       <c r="A31" t="s">
         <v>89</v>
       </c>
@@ -6243,7 +6252,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:28" hidden="1">
+    <row r="32" spans="1:28">
       <c r="A32" t="s">
         <v>90</v>
       </c>
@@ -6327,7 +6336,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:28" hidden="1">
+    <row r="33" spans="1:28">
       <c r="A33" s="2" t="s">
         <v>92</v>
       </c>
@@ -6411,7 +6420,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:28" hidden="1">
+    <row r="34" spans="1:28">
       <c r="A34" s="2" t="s">
         <v>93</v>
       </c>
@@ -6495,7 +6504,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:28" hidden="1">
+    <row r="35" spans="1:28">
       <c r="A35" s="2" t="s">
         <v>94</v>
       </c>
@@ -6579,7 +6588,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:28" hidden="1">
+    <row r="36" spans="1:28">
       <c r="A36" s="2" t="s">
         <v>95</v>
       </c>
@@ -6663,7 +6672,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:28" hidden="1">
+    <row r="37" spans="1:28">
       <c r="A37" s="2" t="s">
         <v>99</v>
       </c>
@@ -6747,7 +6756,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:28" hidden="1">
+    <row r="38" spans="1:28">
       <c r="A38" s="2" t="s">
         <v>100</v>
       </c>
@@ -6831,7 +6840,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:28" hidden="1">
+    <row r="39" spans="1:28">
       <c r="A39" s="2" t="s">
         <v>101</v>
       </c>
@@ -6915,7 +6924,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="40" spans="1:28" hidden="1">
+    <row r="40" spans="1:28">
       <c r="A40" t="s">
         <v>103</v>
       </c>
@@ -6999,7 +7008,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:28" hidden="1">
+    <row r="41" spans="1:28">
       <c r="A41" t="s">
         <v>105</v>
       </c>
@@ -7083,7 +7092,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:28" hidden="1">
+    <row r="42" spans="1:28">
       <c r="A42" s="2" t="s">
         <v>106</v>
       </c>
@@ -7167,7 +7176,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:28" hidden="1">
+    <row r="43" spans="1:28">
       <c r="A43" t="s">
         <v>107</v>
       </c>
@@ -7251,7 +7260,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:28" hidden="1">
+    <row r="44" spans="1:28">
       <c r="A44" s="2" t="s">
         <v>108</v>
       </c>
@@ -7335,7 +7344,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:28" hidden="1">
+    <row r="45" spans="1:28">
       <c r="A45" s="2" t="s">
         <v>110</v>
       </c>
@@ -7419,7 +7428,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:28" hidden="1">
+    <row r="46" spans="1:28">
       <c r="A46" s="2" t="s">
         <v>111</v>
       </c>
@@ -7503,7 +7512,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:28" hidden="1">
+    <row r="47" spans="1:28">
       <c r="A47" s="2" t="s">
         <v>112</v>
       </c>
@@ -7587,7 +7596,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:28" hidden="1">
+    <row r="48" spans="1:28">
       <c r="A48" t="s">
         <v>114</v>
       </c>
@@ -7671,7 +7680,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="49" spans="1:28" hidden="1">
+    <row r="49" spans="1:28">
       <c r="A49" t="s">
         <v>117</v>
       </c>
@@ -7755,7 +7764,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="50" spans="1:28" hidden="1">
+    <row r="50" spans="1:28">
       <c r="A50" t="s">
         <v>118</v>
       </c>
@@ -7839,7 +7848,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="51" spans="1:28" hidden="1">
+    <row r="51" spans="1:28">
       <c r="A51" t="s">
         <v>119</v>
       </c>
@@ -7923,7 +7932,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:28" hidden="1">
+    <row r="52" spans="1:28">
       <c r="A52" t="s">
         <v>120</v>
       </c>
@@ -8007,7 +8016,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:28" hidden="1">
+    <row r="53" spans="1:28">
       <c r="A53" t="s">
         <v>125</v>
       </c>
@@ -8091,7 +8100,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:28" hidden="1">
+    <row r="54" spans="1:28">
       <c r="A54" s="2" t="s">
         <v>126</v>
       </c>
@@ -8175,7 +8184,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:28" hidden="1">
+    <row r="55" spans="1:28">
       <c r="A55" s="2" t="s">
         <v>127</v>
       </c>
@@ -8259,7 +8268,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="56" spans="1:28" hidden="1">
+    <row r="56" spans="1:28">
       <c r="A56" s="2" t="s">
         <v>128</v>
       </c>
@@ -8343,7 +8352,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="1:28" hidden="1">
+    <row r="57" spans="1:28">
       <c r="A57" s="2" t="s">
         <v>132</v>
       </c>
@@ -8427,7 +8436,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:28" hidden="1">
+    <row r="58" spans="1:28">
       <c r="A58" t="s">
         <v>133</v>
       </c>
@@ -8511,7 +8520,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:28" hidden="1">
+    <row r="59" spans="1:28">
       <c r="A59" s="2" t="s">
         <v>134</v>
       </c>
@@ -8595,7 +8604,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:28" hidden="1">
+    <row r="60" spans="1:28">
       <c r="A60" t="s">
         <v>135</v>
       </c>
@@ -8679,7 +8688,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="61" spans="1:28" hidden="1">
+    <row r="61" spans="1:28">
       <c r="A61" t="s">
         <v>138</v>
       </c>
@@ -8763,7 +8772,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="62" spans="1:28" hidden="1">
+    <row r="62" spans="1:28">
       <c r="A62" t="s">
         <v>139</v>
       </c>
@@ -8847,7 +8856,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:28" hidden="1">
+    <row r="63" spans="1:28">
       <c r="A63" t="s">
         <v>140</v>
       </c>
@@ -8931,7 +8940,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="64" spans="1:28" hidden="1">
+    <row r="64" spans="1:28">
       <c r="A64" t="s">
         <v>141</v>
       </c>
@@ -9015,7 +9024,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:28" hidden="1">
+    <row r="65" spans="1:28">
       <c r="A65" t="s">
         <v>144</v>
       </c>
@@ -9183,7 +9192,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="67" spans="1:28" hidden="1">
+    <row r="67" spans="1:28">
       <c r="A67" s="2" t="s">
         <v>149</v>
       </c>
@@ -9267,7 +9276,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="68" spans="1:28" hidden="1">
+    <row r="68" spans="1:28">
       <c r="A68" s="2" t="s">
         <v>150</v>
       </c>
@@ -9351,7 +9360,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="69" spans="1:28" hidden="1">
+    <row r="69" spans="1:28">
       <c r="A69" s="2" t="s">
         <v>151</v>
       </c>
@@ -9435,7 +9444,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:28" hidden="1">
+    <row r="70" spans="1:28">
       <c r="A70" t="s">
         <v>152</v>
       </c>
@@ -9519,7 +9528,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="71" spans="1:28" hidden="1">
+    <row r="71" spans="1:28">
       <c r="A71" t="s">
         <v>154</v>
       </c>
@@ -9603,7 +9612,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:28" hidden="1">
+    <row r="72" spans="1:28">
       <c r="A72" s="2" t="s">
         <v>155</v>
       </c>
@@ -9687,7 +9696,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="73" spans="1:28" hidden="1">
+    <row r="73" spans="1:28">
       <c r="A73" s="2" t="s">
         <v>156</v>
       </c>
@@ -9771,7 +9780,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="74" spans="1:28" hidden="1">
+    <row r="74" spans="1:28">
       <c r="A74" t="s">
         <v>157</v>
       </c>
@@ -9855,7 +9864,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:28" hidden="1">
+    <row r="75" spans="1:28">
       <c r="A75" s="2" t="s">
         <v>159</v>
       </c>
@@ -9939,7 +9948,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="76" spans="1:28" hidden="1">
+    <row r="76" spans="1:28">
       <c r="A76" t="s">
         <v>160</v>
       </c>
@@ -10023,7 +10032,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="77" spans="1:28" hidden="1">
+    <row r="77" spans="1:28">
       <c r="A77" t="s">
         <v>161</v>
       </c>
@@ -10107,7 +10116,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="78" spans="1:28" hidden="1">
+    <row r="78" spans="1:28">
       <c r="A78" t="s">
         <v>162</v>
       </c>
@@ -10191,7 +10200,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="79" spans="1:28" hidden="1">
+    <row r="79" spans="1:28">
       <c r="A79" t="s">
         <v>165</v>
       </c>
@@ -10443,7 +10452,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="82" spans="1:28" hidden="1">
+    <row r="82" spans="1:28">
       <c r="A82" t="s">
         <v>168</v>
       </c>
@@ -10527,7 +10536,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="1:28" hidden="1">
+    <row r="83" spans="1:28">
       <c r="A83" t="s">
         <v>172</v>
       </c>
@@ -10695,7 +10704,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="85" spans="1:28" hidden="1">
+    <row r="85" spans="1:28">
       <c r="A85" s="2" t="s">
         <v>873</v>
       </c>
@@ -10779,7 +10788,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="86" spans="1:28" hidden="1">
+    <row r="86" spans="1:28">
       <c r="A86" s="2" t="s">
         <v>175</v>
       </c>
@@ -10863,7 +10872,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="87" spans="1:28" hidden="1">
+    <row r="87" spans="1:28">
       <c r="A87" s="2" t="s">
         <v>179</v>
       </c>
@@ -10947,7 +10956,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="88" spans="1:28" hidden="1">
+    <row r="88" spans="1:28">
       <c r="A88" s="2" t="s">
         <v>180</v>
       </c>
@@ -11031,7 +11040,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="89" spans="1:28" hidden="1">
+    <row r="89" spans="1:28">
       <c r="A89" t="s">
         <v>181</v>
       </c>
@@ -11115,7 +11124,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="90" spans="1:28" hidden="1">
+    <row r="90" spans="1:28">
       <c r="A90" t="s">
         <v>182</v>
       </c>
@@ -11199,7 +11208,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="91" spans="1:28" hidden="1">
+    <row r="91" spans="1:28">
       <c r="A91" t="s">
         <v>186</v>
       </c>
@@ -11283,7 +11292,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="92" spans="1:28" hidden="1">
+    <row r="92" spans="1:28">
       <c r="A92" t="s">
         <v>187</v>
       </c>
@@ -11367,7 +11376,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="93" spans="1:28" hidden="1">
+    <row r="93" spans="1:28">
       <c r="A93" t="s">
         <v>188</v>
       </c>
@@ -11451,7 +11460,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="94" spans="1:28" hidden="1">
+    <row r="94" spans="1:28">
       <c r="A94" s="2" t="s">
         <v>189</v>
       </c>
@@ -11535,7 +11544,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="95" spans="1:28" hidden="1">
+    <row r="95" spans="1:28">
       <c r="A95" s="2" t="s">
         <v>191</v>
       </c>
@@ -11619,7 +11628,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="96" spans="1:28" hidden="1">
+    <row r="96" spans="1:28">
       <c r="A96" s="2" t="s">
         <v>192</v>
       </c>
@@ -11703,7 +11712,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="97" spans="1:28" hidden="1">
+    <row r="97" spans="1:28">
       <c r="A97" s="2" t="s">
         <v>193</v>
       </c>
@@ -11787,7 +11796,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="98" spans="1:28" hidden="1">
+    <row r="98" spans="1:28">
       <c r="A98" t="s">
         <v>194</v>
       </c>
@@ -11871,7 +11880,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="99" spans="1:28" hidden="1">
+    <row r="99" spans="1:28">
       <c r="A99" s="2" t="s">
         <v>198</v>
       </c>
@@ -11955,7 +11964,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="100" spans="1:28" hidden="1">
+    <row r="100" spans="1:28">
       <c r="A100" t="s">
         <v>199</v>
       </c>
@@ -12039,7 +12048,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="101" spans="1:28" hidden="1">
+    <row r="101" spans="1:28">
       <c r="A101" t="s">
         <v>201</v>
       </c>
@@ -12123,11 +12132,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="102" spans="1:28" hidden="1">
+    <row r="102" spans="1:28">
       <c r="A102" t="s">
         <v>202</v>
       </c>
-      <c r="B102" s="3" t="str">
+      <c r="B102" t="str">
         <f t="shared" si="1"/>
         <v>m-jh1-A-02-07b.txt</v>
       </c>
@@ -12211,7 +12220,7 @@
       <c r="A103" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B103" s="3" t="str">
+      <c r="B103" t="str">
         <f t="shared" si="1"/>
         <v>m-jh1-A-02-07b.txt</v>
       </c>
@@ -12459,7 +12468,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:28" hidden="1">
+    <row r="106" spans="1:28">
       <c r="A106" t="s">
         <v>208</v>
       </c>
@@ -12627,7 +12636,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="108" spans="1:28" hidden="1">
+    <row r="108" spans="1:28">
       <c r="A108" t="s">
         <v>212</v>
       </c>
@@ -12711,7 +12720,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="109" spans="1:28" hidden="1">
+    <row r="109" spans="1:28">
       <c r="A109" t="s">
         <v>213</v>
       </c>
@@ -12879,7 +12888,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:28" hidden="1">
+    <row r="111" spans="1:28">
       <c r="A111" t="s">
         <v>218</v>
       </c>
@@ -12963,7 +12972,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="112" spans="1:28" hidden="1">
+    <row r="112" spans="1:28">
       <c r="A112" t="s">
         <v>219</v>
       </c>
@@ -13047,7 +13056,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="113" spans="1:28" hidden="1">
+    <row r="113" spans="1:28">
       <c r="A113" t="s">
         <v>220</v>
       </c>
@@ -13131,7 +13140,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="114" spans="1:28" hidden="1">
+    <row r="114" spans="1:28">
       <c r="A114" s="2" t="s">
         <v>221</v>
       </c>
@@ -13215,7 +13224,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="115" spans="1:28" hidden="1">
+    <row r="115" spans="1:28">
       <c r="A115" s="2" t="s">
         <v>224</v>
       </c>
@@ -13299,7 +13308,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="116" spans="1:28" hidden="1">
+    <row r="116" spans="1:28">
       <c r="A116" t="s">
         <v>225</v>
       </c>
@@ -13380,7 +13389,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="117" spans="1:28" hidden="1">
+    <row r="117" spans="1:28">
       <c r="A117" t="s">
         <v>229</v>
       </c>
@@ -13461,7 +13470,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="118" spans="1:28" hidden="1">
+    <row r="118" spans="1:28">
       <c r="A118" s="2" t="s">
         <v>230</v>
       </c>
@@ -13545,7 +13554,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="119" spans="1:28" hidden="1">
+    <row r="119" spans="1:28">
       <c r="A119" s="2" t="s">
         <v>237</v>
       </c>
@@ -13629,7 +13638,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="120" spans="1:28" hidden="1">
+    <row r="120" spans="1:28">
       <c r="A120" s="2" t="s">
         <v>238</v>
       </c>
@@ -13713,7 +13722,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="121" spans="1:28" hidden="1">
+    <row r="121" spans="1:28">
       <c r="A121" s="2" t="s">
         <v>239</v>
       </c>
@@ -13797,7 +13806,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="122" spans="1:28" hidden="1">
+    <row r="122" spans="1:28">
       <c r="A122" s="2" t="s">
         <v>240</v>
       </c>
@@ -13881,7 +13890,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="123" spans="1:28" hidden="1">
+    <row r="123" spans="1:28">
       <c r="A123" s="2" t="s">
         <v>242</v>
       </c>
@@ -13965,7 +13974,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="124" spans="1:28" hidden="1">
+    <row r="124" spans="1:28">
       <c r="A124" s="2" t="s">
         <v>243</v>
       </c>
@@ -14049,7 +14058,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="125" spans="1:28" hidden="1">
+    <row r="125" spans="1:28">
       <c r="A125" s="2" t="s">
         <v>244</v>
       </c>
@@ -14133,7 +14142,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="126" spans="1:28" hidden="1">
+    <row r="126" spans="1:28">
       <c r="A126" t="s">
         <v>245</v>
       </c>
@@ -14382,7 +14391,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="129" spans="1:28" hidden="1">
+    <row r="129" spans="1:28">
       <c r="A129" t="s">
         <v>250</v>
       </c>
@@ -14799,7 +14808,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="134" spans="1:28" hidden="1">
+    <row r="134" spans="1:28">
       <c r="A134" t="s">
         <v>255</v>
       </c>
@@ -14880,7 +14889,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="135" spans="1:28" hidden="1">
+    <row r="135" spans="1:28">
       <c r="A135" t="s">
         <v>258</v>
       </c>
@@ -14961,7 +14970,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="136" spans="1:28" hidden="1">
+    <row r="136" spans="1:28">
       <c r="A136" t="s">
         <v>259</v>
       </c>
@@ -15042,7 +15051,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="137" spans="1:28" hidden="1">
+    <row r="137" spans="1:28">
       <c r="A137" t="s">
         <v>260</v>
       </c>
@@ -15123,7 +15132,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="138" spans="1:28" hidden="1">
+    <row r="138" spans="1:28">
       <c r="A138" t="s">
         <v>261</v>
       </c>
@@ -15204,7 +15213,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="139" spans="1:28" hidden="1">
+    <row r="139" spans="1:28">
       <c r="A139" t="s">
         <v>262</v>
       </c>
@@ -15285,7 +15294,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="140" spans="1:28" hidden="1">
+    <row r="140" spans="1:28">
       <c r="A140" t="s">
         <v>263</v>
       </c>
@@ -15366,7 +15375,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="141" spans="1:28" hidden="1">
+    <row r="141" spans="1:28">
       <c r="A141" t="s">
         <v>264</v>
       </c>
@@ -15447,7 +15456,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="142" spans="1:28" hidden="1">
+    <row r="142" spans="1:28">
       <c r="A142" t="s">
         <v>265</v>
       </c>
@@ -15528,7 +15537,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="143" spans="1:28" hidden="1">
+    <row r="143" spans="1:28">
       <c r="A143" t="s">
         <v>268</v>
       </c>
@@ -15609,7 +15618,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="144" spans="1:28" hidden="1">
+    <row r="144" spans="1:28">
       <c r="A144" t="s">
         <v>269</v>
       </c>
@@ -15690,7 +15699,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="145" spans="1:28" hidden="1">
+    <row r="145" spans="1:28">
       <c r="A145" t="s">
         <v>270</v>
       </c>
@@ -15771,7 +15780,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="146" spans="1:28" hidden="1">
+    <row r="146" spans="1:28">
       <c r="A146" t="s">
         <v>271</v>
       </c>
@@ -15852,7 +15861,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="147" spans="1:28" hidden="1">
+    <row r="147" spans="1:28">
       <c r="A147" t="s">
         <v>272</v>
       </c>
@@ -15933,7 +15942,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="148" spans="1:28" hidden="1">
+    <row r="148" spans="1:28">
       <c r="A148" t="s">
         <v>273</v>
       </c>
@@ -16014,7 +16023,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="149" spans="1:28" hidden="1">
+    <row r="149" spans="1:28">
       <c r="A149" t="s">
         <v>274</v>
       </c>
@@ -16095,7 +16104,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="150" spans="1:28" hidden="1">
+    <row r="150" spans="1:28">
       <c r="A150" t="s">
         <v>275</v>
       </c>
@@ -16176,7 +16185,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="151" spans="1:28" hidden="1">
+    <row r="151" spans="1:28">
       <c r="A151" t="s">
         <v>278</v>
       </c>
@@ -16257,7 +16266,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="152" spans="1:28" hidden="1">
+    <row r="152" spans="1:28">
       <c r="A152" t="s">
         <v>279</v>
       </c>
@@ -16422,7 +16431,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="154" spans="1:28" hidden="1">
+    <row r="154" spans="1:28">
       <c r="A154" t="s">
         <v>281</v>
       </c>
@@ -16503,7 +16512,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="155" spans="1:28" hidden="1">
+    <row r="155" spans="1:28">
       <c r="A155" t="s">
         <v>282</v>
       </c>
@@ -16584,7 +16593,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="156" spans="1:28" hidden="1">
+    <row r="156" spans="1:28">
       <c r="A156" t="s">
         <v>283</v>
       </c>
@@ -16665,7 +16674,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="157" spans="1:28" hidden="1">
+    <row r="157" spans="1:28">
       <c r="A157" t="s">
         <v>284</v>
       </c>
@@ -16746,7 +16755,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="158" spans="1:28" hidden="1">
+    <row r="158" spans="1:28">
       <c r="A158" t="s">
         <v>285</v>
       </c>
@@ -16827,7 +16836,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="159" spans="1:28" hidden="1">
+    <row r="159" spans="1:28">
       <c r="A159" t="s">
         <v>289</v>
       </c>
@@ -16908,7 +16917,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="160" spans="1:28" hidden="1">
+    <row r="160" spans="1:28">
       <c r="A160" t="s">
         <v>290</v>
       </c>
@@ -16989,7 +16998,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="161" spans="1:28" hidden="1">
+    <row r="161" spans="1:28">
       <c r="A161" s="2" t="s">
         <v>291</v>
       </c>
@@ -17073,7 +17082,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="162" spans="1:28" hidden="1">
+    <row r="162" spans="1:28">
       <c r="A162" t="s">
         <v>292</v>
       </c>
@@ -17154,7 +17163,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="163" spans="1:28" hidden="1">
+    <row r="163" spans="1:28">
       <c r="A163" t="s">
         <v>293</v>
       </c>
@@ -17235,7 +17244,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="164" spans="1:28" hidden="1">
+    <row r="164" spans="1:28">
       <c r="A164" t="s">
         <v>294</v>
       </c>
@@ -17316,7 +17325,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="165" spans="1:28" hidden="1">
+    <row r="165" spans="1:28">
       <c r="A165" t="s">
         <v>295</v>
       </c>
@@ -17397,7 +17406,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="166" spans="1:28" hidden="1">
+    <row r="166" spans="1:28">
       <c r="A166" t="s">
         <v>296</v>
       </c>
@@ -17478,7 +17487,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="167" spans="1:28" hidden="1">
+    <row r="167" spans="1:28">
       <c r="A167" t="s">
         <v>300</v>
       </c>
@@ -17643,7 +17652,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="169" spans="1:28" hidden="1">
+    <row r="169" spans="1:28">
       <c r="A169" t="s">
         <v>302</v>
       </c>
@@ -17724,7 +17733,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="170" spans="1:28" hidden="1">
+    <row r="170" spans="1:28">
       <c r="A170" t="s">
         <v>303</v>
       </c>
@@ -17805,7 +17814,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="171" spans="1:28" hidden="1">
+    <row r="171" spans="1:28">
       <c r="A171" t="s">
         <v>304</v>
       </c>
@@ -17886,7 +17895,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="172" spans="1:28" hidden="1">
+    <row r="172" spans="1:28">
       <c r="A172" t="s">
         <v>305</v>
       </c>
@@ -17967,7 +17976,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="173" spans="1:28" hidden="1">
+    <row r="173" spans="1:28">
       <c r="A173" t="s">
         <v>306</v>
       </c>
@@ -18048,7 +18057,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="174" spans="1:28" hidden="1">
+    <row r="174" spans="1:28">
       <c r="A174" t="s">
         <v>307</v>
       </c>
@@ -18129,7 +18138,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="175" spans="1:28" hidden="1">
+    <row r="175" spans="1:28">
       <c r="A175" t="s">
         <v>311</v>
       </c>
@@ -18210,7 +18219,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="176" spans="1:28" hidden="1">
+    <row r="176" spans="1:28">
       <c r="A176" t="s">
         <v>312</v>
       </c>
@@ -18291,7 +18300,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="177" spans="1:28" hidden="1">
+    <row r="177" spans="1:28">
       <c r="A177" s="2" t="s">
         <v>313</v>
       </c>
@@ -18459,7 +18468,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="179" spans="1:28" hidden="1">
+    <row r="179" spans="1:28">
       <c r="A179" t="s">
         <v>315</v>
       </c>
@@ -18540,7 +18549,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="180" spans="1:28" hidden="1">
+    <row r="180" spans="1:28">
       <c r="A180" t="s">
         <v>316</v>
       </c>
@@ -18621,7 +18630,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="181" spans="1:28" hidden="1">
+    <row r="181" spans="1:28">
       <c r="A181" t="s">
         <v>317</v>
       </c>
@@ -18702,7 +18711,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="182" spans="1:28" hidden="1">
+    <row r="182" spans="1:28">
       <c r="A182" s="2" t="s">
         <v>318</v>
       </c>
@@ -18786,7 +18795,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="183" spans="1:28" hidden="1">
+    <row r="183" spans="1:28">
       <c r="A183" t="s">
         <v>321</v>
       </c>
@@ -18867,7 +18876,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="184" spans="1:28" hidden="1">
+    <row r="184" spans="1:28">
       <c r="A184" s="2" t="s">
         <v>322</v>
       </c>
@@ -18951,7 +18960,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="185" spans="1:28" hidden="1">
+    <row r="185" spans="1:28">
       <c r="A185" s="2" t="s">
         <v>323</v>
       </c>
@@ -19035,7 +19044,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="186" spans="1:28" hidden="1">
+    <row r="186" spans="1:28">
       <c r="A186" t="s">
         <v>324</v>
       </c>
@@ -19284,7 +19293,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="189" spans="1:28" hidden="1">
+    <row r="189" spans="1:28">
       <c r="A189" s="2" t="s">
         <v>327</v>
       </c>
@@ -19368,7 +19377,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="190" spans="1:28" hidden="1">
+    <row r="190" spans="1:28">
       <c r="A190" s="2" t="s">
         <v>328</v>
       </c>
@@ -19452,7 +19461,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="191" spans="1:28" hidden="1">
+    <row r="191" spans="1:28">
       <c r="A191" s="2" t="s">
         <v>331</v>
       </c>
@@ -19536,7 +19545,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="192" spans="1:28" hidden="1">
+    <row r="192" spans="1:28">
       <c r="A192" s="2" t="s">
         <v>332</v>
       </c>
@@ -19620,7 +19629,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="193" spans="1:28" hidden="1">
+    <row r="193" spans="1:28">
       <c r="A193" s="2" t="s">
         <v>333</v>
       </c>
@@ -19788,7 +19797,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="195" spans="1:28" hidden="1">
+    <row r="195" spans="1:28">
       <c r="A195" s="2" t="s">
         <v>335</v>
       </c>
@@ -19872,7 +19881,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="196" spans="1:28" hidden="1">
+    <row r="196" spans="1:28">
       <c r="A196" s="2" t="s">
         <v>336</v>
       </c>
@@ -19956,7 +19965,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="197" spans="1:28" hidden="1">
+    <row r="197" spans="1:28">
       <c r="A197" s="2" t="s">
         <v>337</v>
       </c>
@@ -20040,7 +20049,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="198" spans="1:28" hidden="1">
+    <row r="198" spans="1:28">
       <c r="A198" t="s">
         <v>338</v>
       </c>
@@ -20121,7 +20130,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="199" spans="1:28" hidden="1">
+    <row r="199" spans="1:28">
       <c r="A199" t="s">
         <v>341</v>
       </c>
@@ -20370,7 +20379,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="202" spans="1:28" hidden="1">
+    <row r="202" spans="1:28">
       <c r="A202" t="s">
         <v>344</v>
       </c>
@@ -20451,7 +20460,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="203" spans="1:28" hidden="1">
+    <row r="203" spans="1:28">
       <c r="A203" t="s">
         <v>345</v>
       </c>
@@ -20616,7 +20625,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="205" spans="1:28" hidden="1">
+    <row r="205" spans="1:28">
       <c r="A205" t="s">
         <v>347</v>
       </c>
@@ -20697,7 +20706,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="206" spans="1:28" hidden="1">
+    <row r="206" spans="1:28">
       <c r="A206" t="s">
         <v>348</v>
       </c>
@@ -20778,7 +20787,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="207" spans="1:28" hidden="1">
+    <row r="207" spans="1:28">
       <c r="A207" t="s">
         <v>353</v>
       </c>
@@ -20859,7 +20868,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="208" spans="1:28" hidden="1">
+    <row r="208" spans="1:28">
       <c r="A208" t="s">
         <v>354</v>
       </c>
@@ -20940,7 +20949,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="209" spans="1:28" hidden="1">
+    <row r="209" spans="1:28">
       <c r="A209" t="s">
         <v>355</v>
       </c>
@@ -21021,7 +21030,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="210" spans="1:28" hidden="1">
+    <row r="210" spans="1:28">
       <c r="A210" t="s">
         <v>356</v>
       </c>
@@ -21102,7 +21111,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="211" spans="1:28" hidden="1">
+    <row r="211" spans="1:28">
       <c r="A211" t="s">
         <v>357</v>
       </c>
@@ -21183,7 +21192,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="212" spans="1:28" hidden="1">
+    <row r="212" spans="1:28">
       <c r="A212" t="s">
         <v>358</v>
       </c>
@@ -21264,7 +21273,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="213" spans="1:28" hidden="1">
+    <row r="213" spans="1:28">
       <c r="A213" t="s">
         <v>359</v>
       </c>
@@ -21345,7 +21354,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="214" spans="1:28" hidden="1">
+    <row r="214" spans="1:28">
       <c r="A214" t="s">
         <v>360</v>
       </c>
@@ -21426,7 +21435,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="215" spans="1:28" hidden="1">
+    <row r="215" spans="1:28">
       <c r="A215" t="s">
         <v>363</v>
       </c>
@@ -21507,7 +21516,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="216" spans="1:28" hidden="1">
+    <row r="216" spans="1:28">
       <c r="A216" t="s">
         <v>364</v>
       </c>
@@ -21588,7 +21597,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="217" spans="1:28" hidden="1">
+    <row r="217" spans="1:28">
       <c r="A217" t="s">
         <v>365</v>
       </c>
@@ -21669,7 +21678,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="218" spans="1:28" hidden="1">
+    <row r="218" spans="1:28">
       <c r="A218" s="2" t="s">
         <v>366</v>
       </c>
@@ -21753,7 +21762,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="219" spans="1:28" hidden="1">
+    <row r="219" spans="1:28">
       <c r="A219" t="s">
         <v>367</v>
       </c>
@@ -21834,7 +21843,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="220" spans="1:28" hidden="1">
+    <row r="220" spans="1:28">
       <c r="A220" s="2" t="s">
         <v>368</v>
       </c>
@@ -21918,7 +21927,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="221" spans="1:28" hidden="1">
+    <row r="221" spans="1:28">
       <c r="A221" t="s">
         <v>369</v>
       </c>
@@ -21999,7 +22008,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="222" spans="1:28" hidden="1">
+    <row r="222" spans="1:28">
       <c r="A222" s="2" t="s">
         <v>370</v>
       </c>
@@ -22083,7 +22092,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="223" spans="1:28" hidden="1">
+    <row r="223" spans="1:28">
       <c r="A223" t="s">
         <v>375</v>
       </c>
@@ -22164,7 +22173,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="224" spans="1:28" hidden="1">
+    <row r="224" spans="1:28">
       <c r="A224" s="2" t="s">
         <v>376</v>
       </c>
@@ -22248,7 +22257,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="225" spans="1:28" hidden="1">
+    <row r="225" spans="1:28">
       <c r="A225" s="2" t="s">
         <v>377</v>
       </c>
@@ -22332,7 +22341,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="226" spans="1:28" hidden="1">
+    <row r="226" spans="1:28">
       <c r="A226" t="s">
         <v>378</v>
       </c>
@@ -22413,7 +22422,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="227" spans="1:28" hidden="1">
+    <row r="227" spans="1:28">
       <c r="A227" t="s">
         <v>379</v>
       </c>
@@ -22494,7 +22503,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="228" spans="1:28" hidden="1">
+    <row r="228" spans="1:28">
       <c r="A228" s="2" t="s">
         <v>380</v>
       </c>
@@ -22578,7 +22587,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="229" spans="1:28" hidden="1">
+    <row r="229" spans="1:28">
       <c r="A229" t="s">
         <v>381</v>
       </c>
@@ -22659,7 +22668,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="230" spans="1:28" hidden="1">
+    <row r="230" spans="1:28">
       <c r="A230" t="s">
         <v>382</v>
       </c>
@@ -22740,7 +22749,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="231" spans="1:28" hidden="1">
+    <row r="231" spans="1:28">
       <c r="A231" t="s">
         <v>387</v>
       </c>
@@ -22821,7 +22830,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="232" spans="1:28" hidden="1">
+    <row r="232" spans="1:28">
       <c r="A232" s="2" t="s">
         <v>388</v>
       </c>
@@ -22905,7 +22914,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="233" spans="1:28" hidden="1">
+    <row r="233" spans="1:28">
       <c r="A233" s="2" t="s">
         <v>389</v>
       </c>
@@ -23073,7 +23082,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="235" spans="1:28" hidden="1">
+    <row r="235" spans="1:28">
       <c r="A235" t="s">
         <v>391</v>
       </c>
@@ -23154,7 +23163,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="236" spans="1:28" hidden="1">
+    <row r="236" spans="1:28">
       <c r="A236" t="s">
         <v>392</v>
       </c>
@@ -23235,7 +23244,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="237" spans="1:28" hidden="1">
+    <row r="237" spans="1:28">
       <c r="A237" t="s">
         <v>393</v>
       </c>
@@ -23316,7 +23325,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="238" spans="1:28" hidden="1">
+    <row r="238" spans="1:28">
       <c r="A238" t="s">
         <v>394</v>
       </c>
@@ -23397,7 +23406,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="239" spans="1:28" hidden="1">
+    <row r="239" spans="1:28">
       <c r="A239" t="s">
         <v>398</v>
       </c>
@@ -23478,7 +23487,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="240" spans="1:28" hidden="1">
+    <row r="240" spans="1:28">
       <c r="A240" t="s">
         <v>399</v>
       </c>
@@ -23559,7 +23568,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="241" spans="1:28" hidden="1">
+    <row r="241" spans="1:28">
       <c r="A241" t="s">
         <v>400</v>
       </c>
@@ -23640,7 +23649,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="242" spans="1:28" hidden="1">
+    <row r="242" spans="1:28">
       <c r="A242" t="s">
         <v>401</v>
       </c>
@@ -23721,7 +23730,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="243" spans="1:28" hidden="1">
+    <row r="243" spans="1:28">
       <c r="A243" t="s">
         <v>402</v>
       </c>
@@ -23886,7 +23895,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="245" spans="1:28" hidden="1">
+    <row r="245" spans="1:28">
       <c r="A245" t="s">
         <v>404</v>
       </c>
@@ -23967,7 +23976,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="246" spans="1:28" hidden="1">
+    <row r="246" spans="1:28">
       <c r="A246" t="s">
         <v>405</v>
       </c>
@@ -24048,7 +24057,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="247" spans="1:28" hidden="1">
+    <row r="247" spans="1:28">
       <c r="A247" t="s">
         <v>407</v>
       </c>
@@ -24129,7 +24138,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="248" spans="1:28" hidden="1">
+    <row r="248" spans="1:28">
       <c r="A248" t="s">
         <v>408</v>
       </c>
@@ -24210,7 +24219,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="249" spans="1:28" hidden="1">
+    <row r="249" spans="1:28">
       <c r="A249" t="s">
         <v>409</v>
       </c>
@@ -24291,7 +24300,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="250" spans="1:28" hidden="1">
+    <row r="250" spans="1:28">
       <c r="A250" t="s">
         <v>410</v>
       </c>
@@ -24372,7 +24381,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="251" spans="1:28" hidden="1">
+    <row r="251" spans="1:28">
       <c r="A251" t="s">
         <v>411</v>
       </c>
@@ -24453,7 +24462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="252" spans="1:28" hidden="1">
+    <row r="252" spans="1:28">
       <c r="A252" t="s">
         <v>412</v>
       </c>
@@ -24534,7 +24543,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="253" spans="1:28" hidden="1">
+    <row r="253" spans="1:28">
       <c r="A253" t="s">
         <v>413</v>
       </c>
@@ -24615,7 +24624,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="254" spans="1:28" hidden="1">
+    <row r="254" spans="1:28">
       <c r="A254" t="s">
         <v>414</v>
       </c>
@@ -24696,7 +24705,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="255" spans="1:28" hidden="1">
+    <row r="255" spans="1:28">
       <c r="A255" t="s">
         <v>416</v>
       </c>
@@ -24777,7 +24786,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="256" spans="1:28" hidden="1">
+    <row r="256" spans="1:28">
       <c r="A256" t="s">
         <v>417</v>
       </c>
@@ -24858,7 +24867,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="257" spans="1:28" hidden="1">
+    <row r="257" spans="1:28">
       <c r="A257" t="s">
         <v>418</v>
       </c>
@@ -24939,7 +24948,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="258" spans="1:28" hidden="1">
+    <row r="258" spans="1:28">
       <c r="A258" t="s">
         <v>419</v>
       </c>
@@ -25020,7 +25029,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="259" spans="1:28" hidden="1">
+    <row r="259" spans="1:28">
       <c r="A259" t="s">
         <v>420</v>
       </c>
@@ -25101,7 +25110,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="260" spans="1:28" hidden="1">
+    <row r="260" spans="1:28">
       <c r="A260" t="s">
         <v>421</v>
       </c>
@@ -25266,7 +25275,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="262" spans="1:28" hidden="1">
+    <row r="262" spans="1:28">
       <c r="A262" t="s">
         <v>423</v>
       </c>
@@ -25347,7 +25356,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="263" spans="1:28" hidden="1">
+    <row r="263" spans="1:28">
       <c r="A263" t="s">
         <v>426</v>
       </c>
@@ -25428,7 +25437,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="264" spans="1:28" hidden="1">
+    <row r="264" spans="1:28">
       <c r="A264" t="s">
         <v>427</v>
       </c>
@@ -25929,7 +25938,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="270" spans="1:28" hidden="1">
+    <row r="270" spans="1:28">
       <c r="A270" t="s">
         <v>433</v>
       </c>
@@ -26010,7 +26019,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="271" spans="1:28" hidden="1">
+    <row r="271" spans="1:28">
       <c r="A271" t="s">
         <v>436</v>
       </c>
@@ -26091,7 +26100,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="272" spans="1:28" hidden="1">
+    <row r="272" spans="1:28">
       <c r="A272" t="s">
         <v>437</v>
       </c>
@@ -26172,7 +26181,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="273" spans="1:28" hidden="1">
+    <row r="273" spans="1:28">
       <c r="A273" t="s">
         <v>438</v>
       </c>
@@ -26253,7 +26262,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="274" spans="1:28" hidden="1">
+    <row r="274" spans="1:28">
       <c r="A274" t="s">
         <v>439</v>
       </c>
@@ -26334,7 +26343,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="275" spans="1:28" hidden="1">
+    <row r="275" spans="1:28">
       <c r="A275" t="s">
         <v>440</v>
       </c>
@@ -26415,7 +26424,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="276" spans="1:28" hidden="1">
+    <row r="276" spans="1:28">
       <c r="A276" t="s">
         <v>441</v>
       </c>
@@ -26496,7 +26505,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="277" spans="1:28" hidden="1">
+    <row r="277" spans="1:28">
       <c r="A277" t="s">
         <v>442</v>
       </c>
@@ -26577,7 +26586,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="278" spans="1:28" hidden="1">
+    <row r="278" spans="1:28">
       <c r="A278" t="s">
         <v>443</v>
       </c>
@@ -26658,7 +26667,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="279" spans="1:28" hidden="1">
+    <row r="279" spans="1:28">
       <c r="A279" t="s">
         <v>446</v>
       </c>
@@ -26739,7 +26748,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="280" spans="1:28" hidden="1">
+    <row r="280" spans="1:28">
       <c r="A280" t="s">
         <v>447</v>
       </c>
@@ -26820,7 +26829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="281" spans="1:28" hidden="1">
+    <row r="281" spans="1:28">
       <c r="A281" t="s">
         <v>448</v>
       </c>
@@ -26901,7 +26910,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="282" spans="1:28" hidden="1">
+    <row r="282" spans="1:28">
       <c r="A282" t="s">
         <v>449</v>
       </c>
@@ -26982,7 +26991,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="283" spans="1:28" hidden="1">
+    <row r="283" spans="1:28">
       <c r="A283" t="s">
         <v>450</v>
       </c>
@@ -27063,7 +27072,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="284" spans="1:28" hidden="1">
+    <row r="284" spans="1:28">
       <c r="A284" t="s">
         <v>451</v>
       </c>
@@ -27144,7 +27153,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="285" spans="1:28" hidden="1">
+    <row r="285" spans="1:28">
       <c r="A285" t="s">
         <v>452</v>
       </c>
@@ -27225,7 +27234,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="286" spans="1:28" hidden="1">
+    <row r="286" spans="1:28">
       <c r="A286" t="s">
         <v>453</v>
       </c>
@@ -27306,7 +27315,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="287" spans="1:28" hidden="1">
+    <row r="287" spans="1:28">
       <c r="A287" t="s">
         <v>456</v>
       </c>
@@ -27387,7 +27396,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="288" spans="1:28" hidden="1">
+    <row r="288" spans="1:28">
       <c r="A288" s="2" t="s">
         <v>457</v>
       </c>
@@ -27471,7 +27480,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="289" spans="1:28" hidden="1">
+    <row r="289" spans="1:28">
       <c r="A289" t="s">
         <v>458</v>
       </c>
@@ -27636,7 +27645,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="291" spans="1:28" hidden="1">
+    <row r="291" spans="1:28">
       <c r="A291" t="s">
         <v>460</v>
       </c>
@@ -27717,7 +27726,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="292" spans="1:28" hidden="1">
+    <row r="292" spans="1:28">
       <c r="A292" t="s">
         <v>461</v>
       </c>
@@ -27798,7 +27807,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="293" spans="1:28" hidden="1">
+    <row r="293" spans="1:28">
       <c r="A293" t="s">
         <v>462</v>
       </c>
@@ -27879,7 +27888,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="294" spans="1:28" hidden="1">
+    <row r="294" spans="1:28">
       <c r="A294" t="s">
         <v>463</v>
       </c>
@@ -27963,7 +27972,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="295" spans="1:28" hidden="1">
+    <row r="295" spans="1:28">
       <c r="A295" s="2" t="s">
         <v>467</v>
       </c>
@@ -28131,7 +28140,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="297" spans="1:28" hidden="1">
+    <row r="297" spans="1:28">
       <c r="A297" s="2" t="s">
         <v>469</v>
       </c>
@@ -28299,7 +28308,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="299" spans="1:28" hidden="1">
+    <row r="299" spans="1:28">
       <c r="A299" t="s">
         <v>471</v>
       </c>
@@ -28380,7 +28389,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="300" spans="1:28" hidden="1">
+    <row r="300" spans="1:28">
       <c r="A300" t="s">
         <v>472</v>
       </c>
@@ -28461,7 +28470,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="301" spans="1:28" hidden="1">
+    <row r="301" spans="1:28">
       <c r="A301" t="s">
         <v>473</v>
       </c>
@@ -28542,7 +28551,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="302" spans="1:28" hidden="1">
+    <row r="302" spans="1:28">
       <c r="A302" t="s">
         <v>474</v>
       </c>
@@ -28623,7 +28632,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="303" spans="1:28" hidden="1">
+    <row r="303" spans="1:28">
       <c r="A303" t="s">
         <v>478</v>
       </c>
@@ -28704,7 +28713,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="304" spans="1:28" hidden="1">
+    <row r="304" spans="1:28">
       <c r="A304" s="2" t="s">
         <v>479</v>
       </c>
@@ -28788,7 +28797,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="305" spans="1:28" hidden="1">
+    <row r="305" spans="1:28">
       <c r="A305" t="s">
         <v>480</v>
       </c>
@@ -28869,7 +28878,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="306" spans="1:28" hidden="1">
+    <row r="306" spans="1:28">
       <c r="A306" t="s">
         <v>481</v>
       </c>
@@ -28950,7 +28959,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="307" spans="1:28" hidden="1">
+    <row r="307" spans="1:28">
       <c r="A307" t="s">
         <v>482</v>
       </c>
@@ -29199,7 +29208,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="310" spans="1:28" hidden="1">
+    <row r="310" spans="1:28">
       <c r="A310" t="s">
         <v>485</v>
       </c>
@@ -29280,7 +29289,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="311" spans="1:28" hidden="1">
+    <row r="311" spans="1:28">
       <c r="A311" t="s">
         <v>487</v>
       </c>
@@ -29361,7 +29370,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="312" spans="1:28" hidden="1">
+    <row r="312" spans="1:28">
       <c r="A312" s="2" t="s">
         <v>488</v>
       </c>
@@ -29445,7 +29454,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="313" spans="1:28" hidden="1">
+    <row r="313" spans="1:28">
       <c r="A313" t="s">
         <v>489</v>
       </c>
@@ -29526,7 +29535,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="314" spans="1:28" hidden="1">
+    <row r="314" spans="1:28">
       <c r="A314" t="s">
         <v>490</v>
       </c>
@@ -29607,7 +29616,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="315" spans="1:28" hidden="1">
+    <row r="315" spans="1:28">
       <c r="A315" s="2" t="s">
         <v>491</v>
       </c>
@@ -29691,7 +29700,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="316" spans="1:28" hidden="1">
+    <row r="316" spans="1:28">
       <c r="A316" t="s">
         <v>492</v>
       </c>
@@ -29772,7 +29781,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="317" spans="1:28" hidden="1">
+    <row r="317" spans="1:28">
       <c r="A317" t="s">
         <v>493</v>
       </c>
@@ -29853,7 +29862,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="318" spans="1:28" hidden="1">
+    <row r="318" spans="1:28">
       <c r="A318" t="s">
         <v>494</v>
       </c>
@@ -29934,7 +29943,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="319" spans="1:28" hidden="1">
+    <row r="319" spans="1:28">
       <c r="A319" t="s">
         <v>497</v>
       </c>
@@ -30015,7 +30024,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="320" spans="1:28" hidden="1">
+    <row r="320" spans="1:28">
       <c r="A320" t="s">
         <v>498</v>
       </c>
@@ -30096,7 +30105,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="321" spans="1:28" hidden="1">
+    <row r="321" spans="1:28">
       <c r="A321" t="s">
         <v>499</v>
       </c>
@@ -30177,7 +30186,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="322" spans="1:28" hidden="1">
+    <row r="322" spans="1:28">
       <c r="A322" t="s">
         <v>500</v>
       </c>
@@ -30258,7 +30267,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="323" spans="1:28" hidden="1">
+    <row r="323" spans="1:28">
       <c r="A323" t="s">
         <v>501</v>
       </c>
@@ -30339,7 +30348,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="324" spans="1:28" hidden="1">
+    <row r="324" spans="1:28">
       <c r="A324" t="s">
         <v>502</v>
       </c>
@@ -30420,7 +30429,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="325" spans="1:28" hidden="1">
+    <row r="325" spans="1:28">
       <c r="A325" t="s">
         <v>503</v>
       </c>
@@ -30501,7 +30510,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="326" spans="1:28" hidden="1">
+    <row r="326" spans="1:28">
       <c r="A326" t="s">
         <v>504</v>
       </c>
@@ -30582,7 +30591,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="327" spans="1:28" hidden="1">
+    <row r="327" spans="1:28">
       <c r="A327" s="2" t="s">
         <v>507</v>
       </c>
@@ -30666,7 +30675,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="328" spans="1:28" hidden="1">
+    <row r="328" spans="1:28">
       <c r="A328" t="s">
         <v>508</v>
       </c>
@@ -30747,7 +30756,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="329" spans="1:28" hidden="1">
+    <row r="329" spans="1:28">
       <c r="A329" t="s">
         <v>509</v>
       </c>
@@ -30828,7 +30837,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="330" spans="1:28" hidden="1">
+    <row r="330" spans="1:28">
       <c r="A330" t="s">
         <v>510</v>
       </c>
@@ -30909,7 +30918,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="331" spans="1:28" hidden="1">
+    <row r="331" spans="1:28">
       <c r="A331" t="s">
         <v>511</v>
       </c>
@@ -30990,7 +30999,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="332" spans="1:28" hidden="1">
+    <row r="332" spans="1:28">
       <c r="A332" t="s">
         <v>512</v>
       </c>
@@ -31071,7 +31080,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="333" spans="1:28" hidden="1">
+    <row r="333" spans="1:28">
       <c r="A333" t="s">
         <v>513</v>
       </c>
@@ -31152,7 +31161,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="334" spans="1:28" hidden="1">
+    <row r="334" spans="1:28">
       <c r="A334" t="s">
         <v>514</v>
       </c>
@@ -31233,7 +31242,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="335" spans="1:28" hidden="1">
+    <row r="335" spans="1:28">
       <c r="A335" t="s">
         <v>516</v>
       </c>
@@ -31314,7 +31323,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="336" spans="1:28" hidden="1">
+    <row r="336" spans="1:28">
       <c r="A336" t="s">
         <v>517</v>
       </c>
@@ -31398,7 +31407,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="337" spans="1:28" hidden="1">
+    <row r="337" spans="1:28">
       <c r="A337" t="s">
         <v>518</v>
       </c>
@@ -31479,7 +31488,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="338" spans="1:28" hidden="1">
+    <row r="338" spans="1:28">
       <c r="A338" t="s">
         <v>519</v>
       </c>
@@ -31560,7 +31569,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="339" spans="1:28" hidden="1">
+    <row r="339" spans="1:28">
       <c r="A339" t="s">
         <v>520</v>
       </c>
@@ -31641,7 +31650,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="340" spans="1:28" hidden="1">
+    <row r="340" spans="1:28">
       <c r="A340" t="s">
         <v>521</v>
       </c>
@@ -31722,7 +31731,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="341" spans="1:28" hidden="1">
+    <row r="341" spans="1:28">
       <c r="A341" t="s">
         <v>522</v>
       </c>
@@ -31803,7 +31812,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="342" spans="1:28" hidden="1">
+    <row r="342" spans="1:28">
       <c r="A342" t="s">
         <v>523</v>
       </c>
@@ -31878,7 +31887,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="343" spans="1:28" hidden="1">
+    <row r="343" spans="1:28">
       <c r="A343" t="s">
         <v>525</v>
       </c>
@@ -32112,7 +32121,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="346" spans="1:28" hidden="1">
+    <row r="346" spans="1:28">
       <c r="A346" t="s">
         <v>528</v>
       </c>
@@ -32187,7 +32196,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="347" spans="1:28" hidden="1">
+    <row r="347" spans="1:28">
       <c r="A347" s="2" t="s">
         <v>529</v>
       </c>
@@ -32265,7 +32274,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="348" spans="1:28" hidden="1">
+    <row r="348" spans="1:28">
       <c r="A348" t="s">
         <v>530</v>
       </c>
@@ -32340,7 +32349,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="349" spans="1:28" hidden="1">
+    <row r="349" spans="1:28">
       <c r="A349" s="2" t="s">
         <v>531</v>
       </c>
@@ -32418,7 +32427,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="350" spans="1:28" hidden="1">
+    <row r="350" spans="1:28">
       <c r="A350" t="s">
         <v>532</v>
       </c>
@@ -32502,7 +32511,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="351" spans="1:28" hidden="1">
+    <row r="351" spans="1:28">
       <c r="A351" t="s">
         <v>541</v>
       </c>
@@ -32586,7 +32595,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="352" spans="1:28" hidden="1">
+    <row r="352" spans="1:28">
       <c r="A352" t="s">
         <v>543</v>
       </c>
@@ -32670,7 +32679,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="353" spans="1:28" hidden="1">
+    <row r="353" spans="1:28">
       <c r="A353" t="s">
         <v>544</v>
       </c>
@@ -32754,7 +32763,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="354" spans="1:28" hidden="1">
+    <row r="354" spans="1:28">
       <c r="A354" t="s">
         <v>546</v>
       </c>
@@ -32838,7 +32847,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="355" spans="1:28" hidden="1">
+    <row r="355" spans="1:28">
       <c r="A355" t="s">
         <v>547</v>
       </c>
@@ -32922,7 +32931,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="356" spans="1:28" hidden="1">
+    <row r="356" spans="1:28">
       <c r="A356" t="s">
         <v>548</v>
       </c>
@@ -33006,7 +33015,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="357" spans="1:28" hidden="1">
+    <row r="357" spans="1:28">
       <c r="A357" t="s">
         <v>551</v>
       </c>
@@ -33090,7 +33099,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="358" spans="1:28" hidden="1">
+    <row r="358" spans="1:28">
       <c r="A358" t="s">
         <v>553</v>
       </c>
@@ -33174,7 +33183,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="359" spans="1:28" hidden="1">
+    <row r="359" spans="1:28">
       <c r="A359" t="s">
         <v>554</v>
       </c>
@@ -33258,7 +33267,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="360" spans="1:28" hidden="1">
+    <row r="360" spans="1:28">
       <c r="A360" t="s">
         <v>555</v>
       </c>
@@ -33342,7 +33351,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="361" spans="1:28" hidden="1">
+    <row r="361" spans="1:28">
       <c r="A361" t="s">
         <v>558</v>
       </c>
@@ -33426,7 +33435,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="362" spans="1:28" hidden="1">
+    <row r="362" spans="1:28">
       <c r="A362" t="s">
         <v>559</v>
       </c>
@@ -33510,7 +33519,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="363" spans="1:28" hidden="1">
+    <row r="363" spans="1:28">
       <c r="A363" t="s">
         <v>560</v>
       </c>
@@ -33594,7 +33603,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="364" spans="1:28" hidden="1">
+    <row r="364" spans="1:28">
       <c r="A364" s="2" t="s">
         <v>561</v>
       </c>
@@ -33678,7 +33687,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="365" spans="1:28" hidden="1">
+    <row r="365" spans="1:28">
       <c r="A365" t="s">
         <v>566</v>
       </c>
@@ -33762,7 +33771,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="366" spans="1:28" hidden="1">
+    <row r="366" spans="1:28">
       <c r="A366" t="s">
         <v>567</v>
       </c>
@@ -33846,7 +33855,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="367" spans="1:28" hidden="1">
+    <row r="367" spans="1:28">
       <c r="A367" t="s">
         <v>568</v>
       </c>
@@ -33930,7 +33939,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="368" spans="1:28" hidden="1">
+    <row r="368" spans="1:28">
       <c r="A368" t="s">
         <v>569</v>
       </c>
@@ -34014,7 +34023,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="369" spans="1:28" hidden="1">
+    <row r="369" spans="1:28">
       <c r="A369" t="s">
         <v>571</v>
       </c>
@@ -34098,7 +34107,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="370" spans="1:28" hidden="1">
+    <row r="370" spans="1:28">
       <c r="A370" t="s">
         <v>572</v>
       </c>
@@ -34182,7 +34191,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="371" spans="1:28" hidden="1">
+    <row r="371" spans="1:28">
       <c r="A371" t="s">
         <v>573</v>
       </c>
@@ -34266,7 +34275,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="372" spans="1:28" hidden="1">
+    <row r="372" spans="1:28">
       <c r="A372" t="s">
         <v>574</v>
       </c>
@@ -34350,7 +34359,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="373" spans="1:28" hidden="1">
+    <row r="373" spans="1:28">
       <c r="A373" t="s">
         <v>576</v>
       </c>
@@ -34434,7 +34443,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="374" spans="1:28" hidden="1">
+    <row r="374" spans="1:28">
       <c r="A374" t="s">
         <v>577</v>
       </c>
@@ -34518,7 +34527,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="375" spans="1:28" hidden="1">
+    <row r="375" spans="1:28">
       <c r="A375" t="s">
         <v>578</v>
       </c>
@@ -34602,7 +34611,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="376" spans="1:28" hidden="1">
+    <row r="376" spans="1:28">
       <c r="A376" t="s">
         <v>579</v>
       </c>
@@ -34686,7 +34695,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="377" spans="1:28" hidden="1">
+    <row r="377" spans="1:28">
       <c r="A377" t="s">
         <v>583</v>
       </c>
@@ -34770,7 +34779,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="378" spans="1:28" hidden="1">
+    <row r="378" spans="1:28">
       <c r="A378" s="2" t="s">
         <v>584</v>
       </c>
@@ -34854,7 +34863,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="379" spans="1:28" hidden="1">
+    <row r="379" spans="1:28">
       <c r="A379" s="2" t="s">
         <v>585</v>
       </c>
@@ -34938,7 +34947,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="380" spans="1:28" hidden="1">
+    <row r="380" spans="1:28">
       <c r="A380" t="s">
         <v>586</v>
       </c>
@@ -35022,7 +35031,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="381" spans="1:28" hidden="1">
+    <row r="381" spans="1:28">
       <c r="A381" t="s">
         <v>588</v>
       </c>
@@ -35106,7 +35115,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="382" spans="1:28" hidden="1">
+    <row r="382" spans="1:28">
       <c r="A382" t="s">
         <v>589</v>
       </c>
@@ -35190,7 +35199,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="383" spans="1:28" hidden="1">
+    <row r="383" spans="1:28">
       <c r="A383" t="s">
         <v>590</v>
       </c>
@@ -35274,7 +35283,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="384" spans="1:28" hidden="1">
+    <row r="384" spans="1:28">
       <c r="A384" t="s">
         <v>591</v>
       </c>
@@ -35358,7 +35367,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="385" spans="1:28" hidden="1">
+    <row r="385" spans="1:28">
       <c r="A385" t="s">
         <v>595</v>
       </c>
@@ -35442,7 +35451,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="386" spans="1:28" hidden="1">
+    <row r="386" spans="1:28">
       <c r="A386" t="s">
         <v>596</v>
       </c>
@@ -35526,7 +35535,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="387" spans="1:28" hidden="1">
+    <row r="387" spans="1:28">
       <c r="A387" t="s">
         <v>597</v>
       </c>
@@ -35610,7 +35619,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="388" spans="1:28" hidden="1">
+    <row r="388" spans="1:28">
       <c r="A388" t="s">
         <v>598</v>
       </c>
@@ -35694,7 +35703,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="389" spans="1:28" hidden="1">
+    <row r="389" spans="1:28">
       <c r="A389" t="s">
         <v>600</v>
       </c>
@@ -35778,7 +35787,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="390" spans="1:28" hidden="1">
+    <row r="390" spans="1:28">
       <c r="A390" t="s">
         <v>601</v>
       </c>
@@ -35862,7 +35871,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="391" spans="1:28" hidden="1">
+    <row r="391" spans="1:28">
       <c r="A391" s="2" t="s">
         <v>602</v>
       </c>
@@ -35946,7 +35955,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="392" spans="1:28" hidden="1">
+    <row r="392" spans="1:28">
       <c r="A392" t="s">
         <v>603</v>
       </c>
@@ -36030,7 +36039,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="393" spans="1:28" hidden="1">
+    <row r="393" spans="1:28">
       <c r="A393" t="s">
         <v>607</v>
       </c>
@@ -36114,7 +36123,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="394" spans="1:28" hidden="1">
+    <row r="394" spans="1:28">
       <c r="A394" s="2" t="s">
         <v>608</v>
       </c>
@@ -36198,7 +36207,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="395" spans="1:28" hidden="1">
+    <row r="395" spans="1:28">
       <c r="A395" t="s">
         <v>609</v>
       </c>
@@ -36282,7 +36291,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="396" spans="1:28" hidden="1">
+    <row r="396" spans="1:28">
       <c r="A396" t="s">
         <v>611</v>
       </c>
@@ -36366,7 +36375,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="397" spans="1:28" hidden="1">
+    <row r="397" spans="1:28">
       <c r="A397" t="s">
         <v>612</v>
       </c>
@@ -36450,7 +36459,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="398" spans="1:28" hidden="1">
+    <row r="398" spans="1:28">
       <c r="A398" t="s">
         <v>614</v>
       </c>
@@ -36534,7 +36543,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="399" spans="1:28" hidden="1">
+    <row r="399" spans="1:28">
       <c r="A399" t="s">
         <v>615</v>
       </c>
@@ -36618,7 +36627,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="400" spans="1:28" hidden="1">
+    <row r="400" spans="1:28">
       <c r="A400" t="s">
         <v>618</v>
       </c>
@@ -36702,7 +36711,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="401" spans="1:28" hidden="1">
+    <row r="401" spans="1:28">
       <c r="A401" t="s">
         <v>619</v>
       </c>
@@ -36786,7 +36795,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="402" spans="1:28" hidden="1">
+    <row r="402" spans="1:28">
       <c r="A402" t="s">
         <v>621</v>
       </c>
@@ -36870,7 +36879,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="403" spans="1:28" hidden="1">
+    <row r="403" spans="1:28">
       <c r="A403" t="s">
         <v>622</v>
       </c>
@@ -36954,7 +36963,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="404" spans="1:28" hidden="1">
+    <row r="404" spans="1:28">
       <c r="A404" t="s">
         <v>624</v>
       </c>
@@ -37038,7 +37047,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="405" spans="1:28" hidden="1">
+    <row r="405" spans="1:28">
       <c r="A405" t="s">
         <v>625</v>
       </c>
@@ -37122,7 +37131,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="406" spans="1:28" hidden="1">
+    <row r="406" spans="1:28">
       <c r="A406" t="s">
         <v>626</v>
       </c>
@@ -37206,7 +37215,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="407" spans="1:28" hidden="1">
+    <row r="407" spans="1:28">
       <c r="A407" t="s">
         <v>627</v>
       </c>
@@ -37290,7 +37299,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="408" spans="1:28" hidden="1">
+    <row r="408" spans="1:28">
       <c r="A408" t="s">
         <v>631</v>
       </c>
@@ -37374,7 +37383,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="409" spans="1:28" hidden="1">
+    <row r="409" spans="1:28">
       <c r="A409" t="s">
         <v>632</v>
       </c>
@@ -37458,7 +37467,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="410" spans="1:28" hidden="1">
+    <row r="410" spans="1:28">
       <c r="A410" t="s">
         <v>633</v>
       </c>
@@ -37542,7 +37551,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="411" spans="1:28" hidden="1">
+    <row r="411" spans="1:28">
       <c r="A411" t="s">
         <v>634</v>
       </c>
@@ -37626,7 +37635,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="412" spans="1:28" hidden="1">
+    <row r="412" spans="1:28">
       <c r="A412" t="s">
         <v>638</v>
       </c>
@@ -37710,7 +37719,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="413" spans="1:28" hidden="1">
+    <row r="413" spans="1:28">
       <c r="A413" t="s">
         <v>639</v>
       </c>
@@ -37794,7 +37803,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="414" spans="1:28" hidden="1">
+    <row r="414" spans="1:28">
       <c r="A414" s="2" t="s">
         <v>640</v>
       </c>
@@ -37878,7 +37887,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="415" spans="1:28" hidden="1">
+    <row r="415" spans="1:28">
       <c r="A415" t="s">
         <v>641</v>
       </c>
@@ -37962,7 +37971,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="416" spans="1:28" hidden="1">
+    <row r="416" spans="1:28">
       <c r="A416" t="s">
         <v>646</v>
       </c>
@@ -38046,7 +38055,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="417" spans="1:28" hidden="1">
+    <row r="417" spans="1:28">
       <c r="A417" s="2" t="s">
         <v>647</v>
       </c>
@@ -38130,7 +38139,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="418" spans="1:28" hidden="1">
+    <row r="418" spans="1:28">
       <c r="A418" t="s">
         <v>648</v>
       </c>
@@ -38214,7 +38223,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="419" spans="1:28" hidden="1">
+    <row r="419" spans="1:28">
       <c r="A419" t="s">
         <v>649</v>
       </c>
@@ -38298,7 +38307,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="420" spans="1:28" hidden="1">
+    <row r="420" spans="1:28">
       <c r="A420" s="2" t="s">
         <v>654</v>
       </c>
@@ -38382,7 +38391,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="421" spans="1:28" hidden="1">
+    <row r="421" spans="1:28">
       <c r="A421" t="s">
         <v>655</v>
       </c>
@@ -38466,7 +38475,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="422" spans="1:28" hidden="1">
+    <row r="422" spans="1:28">
       <c r="A422" t="s">
         <v>656</v>
       </c>
@@ -38550,7 +38559,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="423" spans="1:28" hidden="1">
+    <row r="423" spans="1:28">
       <c r="A423" t="s">
         <v>657</v>
       </c>
@@ -38634,7 +38643,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="424" spans="1:28" hidden="1">
+    <row r="424" spans="1:28">
       <c r="A424" t="s">
         <v>662</v>
       </c>
@@ -38718,7 +38727,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="425" spans="1:28" hidden="1">
+    <row r="425" spans="1:28">
       <c r="A425" t="s">
         <v>663</v>
       </c>
@@ -38802,7 +38811,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="426" spans="1:28" hidden="1">
+    <row r="426" spans="1:28">
       <c r="A426" t="s">
         <v>664</v>
       </c>
@@ -38886,7 +38895,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="427" spans="1:28" hidden="1">
+    <row r="427" spans="1:28">
       <c r="A427" t="s">
         <v>665</v>
       </c>
@@ -38970,7 +38979,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="428" spans="1:28" hidden="1">
+    <row r="428" spans="1:28">
       <c r="A428" t="s">
         <v>667</v>
       </c>
@@ -39054,7 +39063,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="429" spans="1:28" hidden="1">
+    <row r="429" spans="1:28">
       <c r="A429" t="s">
         <v>668</v>
       </c>
@@ -39138,7 +39147,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="430" spans="1:28" hidden="1">
+    <row r="430" spans="1:28">
       <c r="A430" s="2" t="s">
         <v>672</v>
       </c>
@@ -39222,7 +39231,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="431" spans="1:28" hidden="1">
+    <row r="431" spans="1:28">
       <c r="A431" t="s">
         <v>673</v>
       </c>
@@ -39306,7 +39315,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="432" spans="1:28" hidden="1">
+    <row r="432" spans="1:28">
       <c r="A432" s="2" t="s">
         <v>674</v>
       </c>
@@ -39390,7 +39399,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="433" spans="1:28" hidden="1">
+    <row r="433" spans="1:28">
       <c r="A433" t="s">
         <v>676</v>
       </c>
@@ -39474,7 +39483,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="434" spans="1:28" hidden="1">
+    <row r="434" spans="1:28">
       <c r="A434" t="s">
         <v>680</v>
       </c>
@@ -39558,7 +39567,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="435" spans="1:28" hidden="1">
+    <row r="435" spans="1:28">
       <c r="A435" t="s">
         <v>681</v>
       </c>
@@ -39642,7 +39651,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="436" spans="1:28" hidden="1">
+    <row r="436" spans="1:28">
       <c r="A436" t="s">
         <v>682</v>
       </c>
@@ -39726,7 +39735,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="437" spans="1:28" hidden="1">
+    <row r="437" spans="1:28">
       <c r="A437" t="s">
         <v>683</v>
       </c>
@@ -39810,7 +39819,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="438" spans="1:28" hidden="1">
+    <row r="438" spans="1:28">
       <c r="A438" t="s">
         <v>687</v>
       </c>
@@ -39894,7 +39903,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="439" spans="1:28" hidden="1">
+    <row r="439" spans="1:28">
       <c r="A439" t="s">
         <v>688</v>
       </c>
@@ -39978,7 +39987,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="440" spans="1:28" hidden="1">
+    <row r="440" spans="1:28">
       <c r="A440" t="s">
         <v>690</v>
       </c>
@@ -40062,7 +40071,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="441" spans="1:28" hidden="1">
+    <row r="441" spans="1:28">
       <c r="A441" t="s">
         <v>691</v>
       </c>
@@ -40146,7 +40155,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="442" spans="1:28" hidden="1">
+    <row r="442" spans="1:28">
       <c r="A442" t="s">
         <v>694</v>
       </c>
@@ -40230,7 +40239,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="443" spans="1:28" hidden="1">
+    <row r="443" spans="1:28">
       <c r="A443" s="2" t="s">
         <v>695</v>
       </c>
@@ -40314,7 +40323,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="444" spans="1:28" hidden="1">
+    <row r="444" spans="1:28">
       <c r="A444" s="2" t="s">
         <v>696</v>
       </c>
@@ -40398,7 +40407,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="445" spans="1:28" hidden="1">
+    <row r="445" spans="1:28">
       <c r="A445" t="s">
         <v>697</v>
       </c>
@@ -40482,7 +40491,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="446" spans="1:28" hidden="1">
+    <row r="446" spans="1:28">
       <c r="A446" t="s">
         <v>701</v>
       </c>
@@ -40566,7 +40575,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="447" spans="1:28" hidden="1">
+    <row r="447" spans="1:28">
       <c r="A447" t="s">
         <v>702</v>
       </c>
@@ -40650,7 +40659,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="448" spans="1:28" hidden="1">
+    <row r="448" spans="1:28">
       <c r="A448" t="s">
         <v>703</v>
       </c>
@@ -40734,7 +40743,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="449" spans="1:28" hidden="1">
+    <row r="449" spans="1:28">
       <c r="A449" t="s">
         <v>704</v>
       </c>
@@ -40818,7 +40827,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="450" spans="1:28" hidden="1">
+    <row r="450" spans="1:28">
       <c r="A450" t="s">
         <v>708</v>
       </c>
@@ -40902,7 +40911,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="451" spans="1:28" hidden="1">
+    <row r="451" spans="1:28">
       <c r="A451" t="s">
         <v>709</v>
       </c>
@@ -40986,7 +40995,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="452" spans="1:28" hidden="1">
+    <row r="452" spans="1:28">
       <c r="A452" t="s">
         <v>710</v>
       </c>
@@ -41070,7 +41079,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="453" spans="1:28" hidden="1">
+    <row r="453" spans="1:28">
       <c r="A453" t="s">
         <v>711</v>
       </c>
@@ -41154,7 +41163,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="454" spans="1:28" hidden="1">
+    <row r="454" spans="1:28">
       <c r="A454" t="s">
         <v>714</v>
       </c>
@@ -41238,7 +41247,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="455" spans="1:28" hidden="1">
+    <row r="455" spans="1:28">
       <c r="A455" t="s">
         <v>715</v>
       </c>
@@ -41322,7 +41331,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="456" spans="1:28" hidden="1">
+    <row r="456" spans="1:28">
       <c r="A456" t="s">
         <v>716</v>
       </c>
@@ -41406,7 +41415,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="457" spans="1:28" hidden="1">
+    <row r="457" spans="1:28">
       <c r="A457" t="s">
         <v>717</v>
       </c>
@@ -41490,7 +41499,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="458" spans="1:28" hidden="1">
+    <row r="458" spans="1:28">
       <c r="A458" t="s">
         <v>721</v>
       </c>
@@ -41574,7 +41583,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="459" spans="1:28" hidden="1">
+    <row r="459" spans="1:28">
       <c r="A459" t="s">
         <v>722</v>
       </c>
@@ -41658,7 +41667,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="460" spans="1:28" hidden="1">
+    <row r="460" spans="1:28">
       <c r="A460" t="s">
         <v>723</v>
       </c>
@@ -41742,7 +41751,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="461" spans="1:28" hidden="1">
+    <row r="461" spans="1:28">
       <c r="A461" t="s">
         <v>724</v>
       </c>
@@ -41826,7 +41835,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="462" spans="1:28" hidden="1">
+    <row r="462" spans="1:28">
       <c r="A462" t="s">
         <v>728</v>
       </c>
@@ -41910,7 +41919,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="463" spans="1:28" hidden="1">
+    <row r="463" spans="1:28">
       <c r="A463" t="s">
         <v>729</v>
       </c>
@@ -41994,7 +42003,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="464" spans="1:28" hidden="1">
+    <row r="464" spans="1:28">
       <c r="A464" t="s">
         <v>730</v>
       </c>
@@ -42078,7 +42087,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="465" spans="1:28" hidden="1">
+    <row r="465" spans="1:28">
       <c r="A465" s="2" t="s">
         <v>731</v>
       </c>
@@ -42162,7 +42171,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="466" spans="1:28" hidden="1">
+    <row r="466" spans="1:28">
       <c r="A466" t="s">
         <v>734</v>
       </c>
@@ -42246,7 +42255,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="467" spans="1:28" hidden="1">
+    <row r="467" spans="1:28">
       <c r="A467" t="s">
         <v>735</v>
       </c>
@@ -42330,7 +42339,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="468" spans="1:28" hidden="1">
+    <row r="468" spans="1:28">
       <c r="A468" t="s">
         <v>736</v>
       </c>
@@ -42414,7 +42423,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="469" spans="1:28" hidden="1">
+    <row r="469" spans="1:28">
       <c r="A469" s="2" t="s">
         <v>737</v>
       </c>
@@ -42498,7 +42507,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="470" spans="1:28" hidden="1">
+    <row r="470" spans="1:28">
       <c r="A470" t="s">
         <v>741</v>
       </c>
@@ -42582,7 +42591,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="471" spans="1:28" hidden="1">
+    <row r="471" spans="1:28">
       <c r="A471" s="2" t="s">
         <v>742</v>
       </c>
@@ -42666,7 +42675,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="472" spans="1:28" hidden="1">
+    <row r="472" spans="1:28">
       <c r="A472" s="2" t="s">
         <v>743</v>
       </c>
@@ -42750,7 +42759,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="473" spans="1:28" hidden="1">
+    <row r="473" spans="1:28">
       <c r="A473" s="2" t="s">
         <v>744</v>
       </c>
@@ -42834,7 +42843,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="474" spans="1:28" hidden="1">
+    <row r="474" spans="1:28">
       <c r="A474" t="s">
         <v>748</v>
       </c>
@@ -42918,7 +42927,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="475" spans="1:28" hidden="1">
+    <row r="475" spans="1:28">
       <c r="A475" t="s">
         <v>749</v>
       </c>
@@ -43002,7 +43011,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="476" spans="1:28" hidden="1">
+    <row r="476" spans="1:28">
       <c r="A476" s="2" t="s">
         <v>750</v>
       </c>
@@ -43086,7 +43095,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="477" spans="1:28" hidden="1">
+    <row r="477" spans="1:28">
       <c r="A477" t="s">
         <v>751</v>
       </c>
@@ -43170,7 +43179,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="478" spans="1:28" hidden="1">
+    <row r="478" spans="1:28">
       <c r="A478" t="s">
         <v>754</v>
       </c>
@@ -43254,7 +43263,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="479" spans="1:28" hidden="1">
+    <row r="479" spans="1:28">
       <c r="A479" t="s">
         <v>755</v>
       </c>
@@ -43338,7 +43347,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="480" spans="1:28" hidden="1">
+    <row r="480" spans="1:28">
       <c r="A480" s="2" t="s">
         <v>757</v>
       </c>
@@ -43422,7 +43431,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="481" spans="1:28" hidden="1">
+    <row r="481" spans="1:28">
       <c r="A481" t="s">
         <v>758</v>
       </c>
@@ -43506,7 +43515,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="482" spans="1:28" hidden="1">
+    <row r="482" spans="1:28">
       <c r="A482" t="s">
         <v>760</v>
       </c>
@@ -43590,7 +43599,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="483" spans="1:28" hidden="1">
+    <row r="483" spans="1:28">
       <c r="A483" s="2" t="s">
         <v>761</v>
       </c>
@@ -43674,7 +43683,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="484" spans="1:28" hidden="1">
+    <row r="484" spans="1:28">
       <c r="A484" s="2" t="s">
         <v>763</v>
       </c>
@@ -43758,7 +43767,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="485" spans="1:28" hidden="1">
+    <row r="485" spans="1:28">
       <c r="A485" t="s">
         <v>764</v>
       </c>
@@ -43842,7 +43851,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="486" spans="1:28" hidden="1">
+    <row r="486" spans="1:28">
       <c r="A486" t="s">
         <v>767</v>
       </c>
@@ -43926,7 +43935,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="487" spans="1:28" hidden="1">
+    <row r="487" spans="1:28">
       <c r="A487" s="2" t="s">
         <v>768</v>
       </c>
@@ -44010,7 +44019,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="488" spans="1:28" hidden="1">
+    <row r="488" spans="1:28">
       <c r="A488" s="2" t="s">
         <v>770</v>
       </c>
@@ -44094,7 +44103,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="489" spans="1:28" hidden="1">
+    <row r="489" spans="1:28">
       <c r="A489" s="2" t="s">
         <v>771</v>
       </c>
@@ -44178,7 +44187,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="490" spans="1:28" hidden="1">
+    <row r="490" spans="1:28">
       <c r="A490" s="2" t="s">
         <v>774</v>
       </c>
@@ -44262,7 +44271,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="491" spans="1:28" hidden="1">
+    <row r="491" spans="1:28">
       <c r="A491" s="2" t="s">
         <v>775</v>
       </c>
@@ -44346,7 +44355,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="492" spans="1:28" hidden="1">
+    <row r="492" spans="1:28">
       <c r="A492" s="2" t="s">
         <v>776</v>
       </c>
@@ -44430,7 +44439,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="493" spans="1:28" hidden="1">
+    <row r="493" spans="1:28">
       <c r="A493" s="2" t="s">
         <v>777</v>
       </c>
@@ -44514,7 +44523,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="494" spans="1:28" hidden="1">
+    <row r="494" spans="1:28">
       <c r="A494" t="s">
         <v>782</v>
       </c>
@@ -44598,7 +44607,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="495" spans="1:28" hidden="1">
+    <row r="495" spans="1:28">
       <c r="A495" s="2" t="s">
         <v>783</v>
       </c>
@@ -44682,7 +44691,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="496" spans="1:28" hidden="1">
+    <row r="496" spans="1:28">
       <c r="A496" t="s">
         <v>788</v>
       </c>
@@ -44766,7 +44775,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="497" spans="1:28" hidden="1">
+    <row r="497" spans="1:28">
       <c r="A497" s="2" t="s">
         <v>789</v>
       </c>
@@ -44850,7 +44859,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="498" spans="1:28" hidden="1">
+    <row r="498" spans="1:28">
       <c r="A498" s="2" t="s">
         <v>791</v>
       </c>
@@ -44934,7 +44943,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="499" spans="1:28" hidden="1">
+    <row r="499" spans="1:28">
       <c r="A499" s="2" t="s">
         <v>865</v>
       </c>
@@ -45018,7 +45027,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="500" spans="1:28" hidden="1">
+    <row r="500" spans="1:28">
       <c r="A500" s="2" t="s">
         <v>796</v>
       </c>
@@ -45102,7 +45111,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="501" spans="1:28" hidden="1">
+    <row r="501" spans="1:28">
       <c r="A501" s="2" t="s">
         <v>797</v>
       </c>
@@ -45186,7 +45195,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="502" spans="1:28" hidden="1">
+    <row r="502" spans="1:28">
       <c r="A502" s="2" t="s">
         <v>798</v>
       </c>
@@ -45270,7 +45279,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="503" spans="1:28" hidden="1">
+    <row r="503" spans="1:28">
       <c r="A503" t="s">
         <v>799</v>
       </c>
@@ -45354,7 +45363,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="504" spans="1:28" hidden="1">
+    <row r="504" spans="1:28">
       <c r="A504" s="2" t="s">
         <v>803</v>
       </c>
@@ -45438,7 +45447,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="505" spans="1:28" hidden="1">
+    <row r="505" spans="1:28">
       <c r="A505" s="2" t="s">
         <v>804</v>
       </c>
@@ -45522,7 +45531,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="506" spans="1:28" hidden="1">
+    <row r="506" spans="1:28">
       <c r="A506" s="2" t="s">
         <v>806</v>
       </c>
@@ -45606,7 +45615,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="507" spans="1:28" hidden="1">
+    <row r="507" spans="1:28">
       <c r="A507" s="2" t="s">
         <v>807</v>
       </c>
@@ -45690,7 +45699,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="508" spans="1:28" hidden="1">
+    <row r="508" spans="1:28">
       <c r="A508" t="s">
         <v>811</v>
       </c>
@@ -45774,7 +45783,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="509" spans="1:28" hidden="1">
+    <row r="509" spans="1:28">
       <c r="A509" s="2" t="s">
         <v>812</v>
       </c>
@@ -45858,7 +45867,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="510" spans="1:28" hidden="1">
+    <row r="510" spans="1:28">
       <c r="A510" t="s">
         <v>815</v>
       </c>
@@ -45942,7 +45951,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="511" spans="1:28" hidden="1">
+    <row r="511" spans="1:28">
       <c r="A511" t="s">
         <v>816</v>
       </c>
@@ -46026,7 +46035,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="512" spans="1:28" hidden="1">
+    <row r="512" spans="1:28">
       <c r="A512" t="s">
         <v>819</v>
       </c>
@@ -46110,7 +46119,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="513" spans="1:28" hidden="1">
+    <row r="513" spans="1:28">
       <c r="A513" t="s">
         <v>820</v>
       </c>
@@ -46194,7 +46203,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="514" spans="1:28" hidden="1">
+    <row r="514" spans="1:28">
       <c r="A514" t="s">
         <v>863</v>
       </c>
@@ -46281,7 +46290,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="515" spans="1:28" hidden="1">
+    <row r="515" spans="1:28">
       <c r="A515" t="s">
         <v>825</v>
       </c>
@@ -46365,7 +46374,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="516" spans="1:28" hidden="1">
+    <row r="516" spans="1:28">
       <c r="A516" t="s">
         <v>829</v>
       </c>
@@ -46449,7 +46458,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="517" spans="1:28" hidden="1">
+    <row r="517" spans="1:28">
       <c r="A517" s="2" t="s">
         <v>830</v>
       </c>
@@ -46533,7 +46542,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="518" spans="1:28" hidden="1">
+    <row r="518" spans="1:28">
       <c r="A518" s="2" t="s">
         <v>831</v>
       </c>
@@ -46617,7 +46626,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="519" spans="1:28" hidden="1">
+    <row r="519" spans="1:28">
       <c r="A519" s="2" t="s">
         <v>832</v>
       </c>
@@ -46701,7 +46710,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="520" spans="1:28" hidden="1">
+    <row r="520" spans="1:28">
       <c r="A520" t="s">
         <v>836</v>
       </c>
@@ -46785,7 +46794,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="521" spans="1:28" hidden="1">
+    <row r="521" spans="1:28">
       <c r="A521" s="2" t="s">
         <v>837</v>
       </c>
@@ -46869,7 +46878,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="522" spans="1:28" hidden="1">
+    <row r="522" spans="1:28">
       <c r="A522" t="s">
         <v>838</v>
       </c>
@@ -46953,7 +46962,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="523" spans="1:28" hidden="1">
+    <row r="523" spans="1:28">
       <c r="A523" t="s">
         <v>839</v>
       </c>
@@ -47037,7 +47046,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="524" spans="1:28" hidden="1">
+    <row r="524" spans="1:28">
       <c r="A524" s="2" t="s">
         <v>843</v>
       </c>
@@ -47121,7 +47130,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="525" spans="1:28" hidden="1">
+    <row r="525" spans="1:28">
       <c r="A525" s="2" t="s">
         <v>844</v>
       </c>
@@ -47205,7 +47214,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="526" spans="1:28" hidden="1">
+    <row r="526" spans="1:28">
       <c r="A526" s="2" t="s">
         <v>845</v>
       </c>
@@ -47289,7 +47298,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="527" spans="1:28" hidden="1">
+    <row r="527" spans="1:28">
       <c r="A527" s="2" t="s">
         <v>846</v>
       </c>
@@ -47373,7 +47382,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="528" spans="1:28" hidden="1">
+    <row r="528" spans="1:28">
       <c r="A528" t="s">
         <v>849</v>
       </c>
@@ -47457,7 +47466,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="529" spans="1:28" hidden="1">
+    <row r="529" spans="1:28">
       <c r="A529" s="2" t="s">
         <v>850</v>
       </c>
@@ -47541,7 +47550,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="530" spans="1:28" hidden="1">
+    <row r="530" spans="1:28">
       <c r="A530" s="2" t="s">
         <v>851</v>
       </c>
@@ -47625,7 +47634,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="531" spans="1:28" hidden="1">
+    <row r="531" spans="1:28">
       <c r="A531" s="2" t="s">
         <v>853</v>
       </c>
@@ -47709,7 +47718,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="532" spans="1:28" hidden="1">
+    <row r="532" spans="1:28">
       <c r="A532" s="2" t="s">
         <v>856</v>
       </c>
@@ -47793,7 +47802,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="533" spans="1:28" hidden="1">
+    <row r="533" spans="1:28">
       <c r="A533" s="2" t="s">
         <v>857</v>
       </c>
@@ -47877,7 +47886,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="534" spans="1:28" hidden="1">
+    <row r="534" spans="1:28">
       <c r="A534" s="2" t="s">
         <v>858</v>
       </c>
@@ -47962,14 +47971,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB1048576" xr:uid="{04D504C1-10AA-394B-B3F6-5620CD148B80}">
-    <filterColumn colId="27">
-      <filters>
-        <filter val="必要に応じて間違えやすい点を1文添える"/>
-        <filter val="必要に応じて間違えやすい点を1文添える；"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AB1048576" xr:uid="{04D504C1-10AA-394B-B3F6-5620CD148B80}"/>
   <phoneticPr fontId="18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>